<commit_message>
chore(historicos): update Excels from local BEVSA run 2026-02-24
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/update/historicos/HistoricoDiario.xlsx
+++ b/update/historicos/HistoricoDiario.xlsx
@@ -189,7 +189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr customHeight="false" defaultColWidth="9.28125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -226,548 +226,522 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46059</v>
+        <v>46077</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>38.516</v>
+        <v>38.397</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>38.516</v>
+        <v>38.397</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>38.56</v>
+        <v>38.39</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>38.55</v>
+        <v>38.39</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>38.6</v>
+        <v>38.4</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>35000000</v>
+        <v>27000000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46058</v>
+        <v>46076</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>38.776</v>
+        <v>38.353</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>38.776</v>
+        <v>38.353</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>38.68</v>
+        <v>38.45</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>38.65</v>
+        <v>38.4</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>38.72</v>
+        <v>38.48</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>33300000</v>
+        <v>41300000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46057</v>
+        <v>46073</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>38.641</v>
+        <v>38.708</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>38.641</v>
+        <v>38.708</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>38.75</v>
+        <v>38.5</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>38.7</v>
+        <v>38.4</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>38.8</v>
+        <v>38.6</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>30000000</v>
+        <v>24600000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46056</v>
+        <v>46072</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>38.566</v>
+        <v>38.76</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>38.566</v>
+        <v>38.76</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>38.58</v>
+        <v>38.85</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>38.57</v>
+        <v>38.78</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>38.59</v>
+        <v>38.9</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>23500000</v>
+        <v>34500000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46055</v>
+        <v>46071</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>38.523</v>
+        <v>38.79</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>38.523</v>
+        <v>38.79</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>38.57</v>
+        <v>38.76</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>38.55</v>
+        <v>38.74</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>38.6</v>
+        <v>38.79</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>46500000</v>
+        <v>36000000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46052</v>
+        <v>46066</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>38.5</v>
+        <v>38.841</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>38.5</v>
+        <v>38.841</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>38.52</v>
+        <v>38.87</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>38.48</v>
+        <v>38.83</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>38.53</v>
+        <v>38.95</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>38800000</v>
+        <v>21000000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46051</v>
+        <v>46065</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>38.784</v>
+        <v>38.731</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>38.784</v>
+        <v>38.731</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>38.65</v>
+        <v>38.75</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>38.6</v>
+        <v>38.74</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>38.75</v>
+        <v>38.76</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>59800000</v>
+        <v>46600000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46050</v>
+        <v>46064</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>38.793</v>
+        <v>38.537</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>38.793</v>
+        <v>38.537</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>38.9</v>
+        <v>38.65</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>38.87</v>
+        <v>38.62</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>38.95</v>
+        <v>38.75</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>25400000</v>
+        <v>29000000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46049</v>
+        <v>46063</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>37.983</v>
+        <v>38.469</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>37.983</v>
+        <v>38.469</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>38.3</v>
+        <v>38.48</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>38.2</v>
+        <v>38.45</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>38.45</v>
+        <v>38.49</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>40200000</v>
+        <v>14500000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46048</v>
+        <v>46062</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>37.831</v>
+        <v>38.364</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>37.831</v>
+        <v>38.364</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>37.8</v>
+        <v>38.4</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>37.73</v>
+        <v>38.38</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>37.82</v>
+        <v>38.44</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>121</v>
+        <v>78</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>63000000</v>
+        <v>44000000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46045</v>
+        <v>46059</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>37.454</v>
+        <v>38.516</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>37.454</v>
+        <v>38.516</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>38</v>
+        <v>38.56</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>38</v>
+        <v>38.55</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>38.15</v>
+        <v>38.6</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>163</v>
+        <v>70</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>83100000</v>
+        <v>35000000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46044</v>
+        <v>46058</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>37.512</v>
+        <v>38.776</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>37.512</v>
+        <v>38.776</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>37.3</v>
+        <v>38.68</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>37.25</v>
+        <v>38.65</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>37.35</v>
+        <v>38.72</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>26400000</v>
+        <v>33300000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46043</v>
+        <v>46057</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>37.854</v>
+        <v>38.641</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>37.854</v>
+        <v>38.641</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>37.8</v>
+        <v>38.75</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>37.75</v>
+        <v>38.7</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>37.85</v>
+        <v>38.8</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="H15" s="1" t="n">
-        <v>35700000</v>
+        <v>30000000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46042</v>
+        <v>46056</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>38.218</v>
+        <v>38.566</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>38.218</v>
+        <v>38.566</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>38.18</v>
+        <v>38.58</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>38.18</v>
+        <v>38.57</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>38.22</v>
+        <v>38.59</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>37500000</v>
+        <v>23500000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46041</v>
+        <v>46055</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>38.349</v>
+        <v>38.523</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>38.349</v>
+        <v>38.523</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>38.31</v>
+        <v>38.57</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>38.31</v>
+        <v>38.55</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>38.34</v>
+        <v>38.6</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>11000000</v>
+        <v>46500000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46038</v>
+        <v>46052</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>38.415</v>
+        <v>38.5</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>38.415</v>
+        <v>38.5</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>38.45</v>
+        <v>38.52</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>38.4</v>
+        <v>38.48</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>38.45</v>
+        <v>38.53</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="H18" s="1" t="n">
-        <v>22000000</v>
+        <v>38800000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46037</v>
+        <v>46051</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>38.599</v>
+        <v>38.784</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>38.599</v>
+        <v>38.784</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>38.55</v>
+        <v>38.65</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>38.51</v>
+        <v>38.6</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>38.55</v>
+        <v>38.75</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>18500000</v>
+        <v>59800000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46036</v>
+        <v>46050</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>38.685</v>
+        <v>38.793</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>38.685</v>
+        <v>38.793</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>38.65</v>
+        <v>38.9</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>38.62</v>
+        <v>38.87</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>38.65</v>
+        <v>38.95</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>28900000</v>
+        <v>25400000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46035</v>
+        <v>46049</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>38.597</v>
+        <v>37.983</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>38.597</v>
+        <v>37.983</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>38.7</v>
+        <v>38.3</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>38.7</v>
+        <v>38.2</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>38.75</v>
+        <v>38.45</v>
       </c>
       <c r="G21" s="1" t="n">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>33500000</v>
+        <v>40200000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46034</v>
+        <v>46048</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>38.72</v>
+        <v>37.831</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>38.72</v>
+        <v>37.831</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>38.68</v>
+        <v>37.8</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>38.65</v>
+        <v>37.73</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>38.73</v>
+        <v>37.82</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="H22" s="1" t="n">
-        <v>33000000</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>46031</v>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>38.815</v>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>38.815</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>38.79</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>38.79</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>38.82</v>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>38</v>
-      </c>
-      <c r="H23" s="1" t="n">
-        <v>19000000</v>
+        <v>63000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>